<commit_message>
Update seminar data pipeline for v4 events
</commit_message>
<xml_diff>
--- a/outputs/analysis/tables/event_study_panel_summary_baseline_minus1.xlsx
+++ b/outputs/analysis/tables/event_study_panel_summary_baseline_minus1.xlsx
@@ -62,17 +62,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>-0.081***</t>
+          <t>-0.041</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>-0.091</t>
+          <t>0.218</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>-0.057**</t>
+          <t>-0.086</t>
         </is>
       </c>
     </row>
@@ -84,17 +84,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>(0.027)</t>
+          <t>(0.064)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>(0.101)</t>
+          <t>(0.177)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>(0.027)</t>
+          <t>(0.069)</t>
         </is>
       </c>
     </row>
@@ -128,17 +128,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>-0.215***</t>
+          <t>-0.071</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>-0.359</t>
+          <t>0.415*</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>-0.164***</t>
+          <t>-0.158*</t>
         </is>
       </c>
     </row>
@@ -150,17 +150,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>(0.047)</t>
+          <t>(0.082)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>(0.228)</t>
+          <t>(0.231)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>(0.044)</t>
+          <t>(0.085)</t>
         </is>
       </c>
     </row>
@@ -194,17 +194,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0.075*</t>
+          <t>-0.059</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>0.174*</t>
+          <t>0.017</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0.069*</t>
+          <t>-0.058</t>
         </is>
       </c>
     </row>
@@ -216,17 +216,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>(0.038)</t>
+          <t>(0.085)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>(0.085)</t>
+          <t>(0.193)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>(0.039)</t>
+          <t>(0.093)</t>
         </is>
       </c>
     </row>
@@ -260,17 +260,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>0.347</t>
+          <t>0.357</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>0.436</t>
+          <t>0.369</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.362</t>
+          <t>0.373</t>
         </is>
       </c>
     </row>
@@ -282,17 +282,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0.329</t>
+          <t>0.353</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0.454</t>
+          <t>0.415</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>0.342</t>
+          <t>0.357</t>
         </is>
       </c>
     </row>
@@ -304,17 +304,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>0.407</t>
+          <t>0.521</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>0.483</t>
+          <t>0.486</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>0.415</t>
+          <t>0.538</t>
         </is>
       </c>
     </row>
@@ -348,12 +348,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>9,458</t>
+          <t>9,548</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>1,539</t>
+          <t>1,629</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -370,17 +370,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>10,038</t>
+          <t>1,825</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>1,411</t>
+          <t>253</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>8,627</t>
+          <t>1,572</t>
         </is>
       </c>
     </row>
@@ -392,17 +392,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>5,543</t>
+          <t>1,658</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>817</t>
+          <t>242</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>4,726</t>
+          <t>1,416</t>
         </is>
       </c>
     </row>
@@ -414,17 +414,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>5,323</t>
+          <t>1,039</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>755</t>
+          <t>180</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>4,568</t>
+          <t>859</t>
         </is>
       </c>
     </row>
@@ -436,17 +436,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>4,090</t>
+          <t>928</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>599</t>
+          <t>169</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>3,491</t>
+          <t>759</t>
         </is>
       </c>
     </row>
@@ -458,17 +458,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>4,714</t>
+          <t>784</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>656</t>
+          <t>73</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>4,058</t>
+          <t>711</t>
         </is>
       </c>
     </row>
@@ -480,17 +480,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>3,391</t>
+          <t>730</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>470</t>
+          <t>73</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2,921</t>
+          <t>657</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Normalize significance codes to R defaults
</commit_message>
<xml_diff>
--- a/outputs/analysis/tables/event_study_panel_summary_baseline_minus1.xlsx
+++ b/outputs/analysis/tables/event_study_panel_summary_baseline_minus1.xlsx
@@ -133,12 +133,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>0.415*</t>
+          <t>0.415.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>-0.158*</t>
+          <t>-0.158.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add paper-ready sample statistics table outputs
</commit_message>
<xml_diff>
--- a/outputs/analysis/tables/event_study_panel_summary_baseline_minus1.xlsx
+++ b/outputs/analysis/tables/event_study_panel_summary_baseline_minus1.xlsx
@@ -62,17 +62,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>-0.041</t>
+          <t>-0.032</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0.218</t>
+          <t>0.132</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>-0.086</t>
+          <t>-0.060</t>
         </is>
       </c>
     </row>
@@ -84,17 +84,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>(0.064)</t>
+          <t>(0.041)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>(0.177)</t>
+          <t>(0.122)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>(0.069)</t>
+          <t>(0.044)</t>
         </is>
       </c>
     </row>
@@ -128,17 +128,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>-0.071</t>
+          <t>-0.065</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>0.415.</t>
+          <t>0.379.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>-0.158.</t>
+          <t>-0.145.</t>
         </is>
       </c>
     </row>
@@ -150,17 +150,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>(0.082)</t>
+          <t>(0.077)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>(0.231)</t>
+          <t>(0.204)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>(0.085)</t>
+          <t>(0.078)</t>
         </is>
       </c>
     </row>
@@ -194,17 +194,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>-0.059</t>
+          <t>-0.014</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>0.017</t>
+          <t>0.053</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>-0.058</t>
+          <t>-0.021</t>
         </is>
       </c>
     </row>
@@ -216,17 +216,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>(0.085)</t>
+          <t>(0.053)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>(0.193)</t>
+          <t>(0.178)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>(0.093)</t>
+          <t>(0.056)</t>
         </is>
       </c>
     </row>
@@ -260,17 +260,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>0.357</t>
+          <t>0.398</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>0.369</t>
+          <t>0.433</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.373</t>
+          <t>0.413</t>
         </is>
       </c>
     </row>
@@ -282,17 +282,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0.353</t>
+          <t>0.369</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0.415</t>
+          <t>0.416</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>0.357</t>
+          <t>0.387</t>
         </is>
       </c>
     </row>
@@ -304,17 +304,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>0.521</t>
+          <t>0.463</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>0.486</t>
+          <t>0.506</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>0.538</t>
+          <t>0.467</t>
         </is>
       </c>
     </row>
@@ -370,17 +370,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>1,825</t>
+          <t>3,887</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>253</t>
+          <t>567</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>1,572</t>
+          <t>3,320</t>
         </is>
       </c>
     </row>
@@ -392,17 +392,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>1,658</t>
+          <t>2,925</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>242</t>
+          <t>412</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>1,416</t>
+          <t>2,513</t>
         </is>
       </c>
     </row>
@@ -414,17 +414,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>1,039</t>
+          <t>1,373</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>215</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>859</t>
+          <t>1,158</t>
         </is>
       </c>
     </row>
@@ -436,17 +436,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>928</t>
+          <t>1,261</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>169</t>
+          <t>204</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>759</t>
+          <t>1,057</t>
         </is>
       </c>
     </row>
@@ -458,17 +458,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>784</t>
+          <t>2,512</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>73</t>
+          <t>352</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>711</t>
+          <t>2,160</t>
         </is>
       </c>
     </row>
@@ -480,17 +480,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>730</t>
+          <t>2,073</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>73</t>
+          <t>271</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>657</t>
+          <t>1,802</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Harden Meta USD conversion secrets handling
</commit_message>
<xml_diff>
--- a/outputs/analysis/tables/event_study_panel_summary_baseline_minus1.xlsx
+++ b/outputs/analysis/tables/event_study_panel_summary_baseline_minus1.xlsx
@@ -314,7 +314,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>0.467</t>
+          <t>0.466</t>
         </is>
       </c>
     </row>
@@ -348,7 +348,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>9,548</t>
+          <t>9,549</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -358,7 +358,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>7,919</t>
+          <t>7,920</t>
         </is>
       </c>
     </row>

</xml_diff>